<commit_message>
Removendo banco de dados do versionamento
</commit_message>
<xml_diff>
--- a/database/lojas e senhas.xlsx
+++ b/database/lojas e senhas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Desktop\TeleFluxo_Instalador\database\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF499FCA-019A-4EDD-8DE3-FFDD4B2EA75B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B79FBF8-9A16-4B7E-9978-5C2339763BDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{DC387A1A-0365-4EFE-8541-627FD66421E4}"/>
   </bookViews>
@@ -412,7 +412,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -437,12 +437,6 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -870,7 +864,7 @@
       <c r="F5" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="H5" s="10" t="s">
+      <c r="H5" s="7" t="s">
         <v>84</v>
       </c>
     </row>
@@ -893,7 +887,7 @@
       <c r="F6" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="H6" s="11" t="s">
+      <c r="H6" s="9" t="s">
         <v>84</v>
       </c>
     </row>
@@ -976,7 +970,7 @@
       <c r="F10" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="H10" s="10" t="s">
+      <c r="H10" s="7" t="s">
         <v>85</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Ajustes e upgrade sacolas
</commit_message>
<xml_diff>
--- a/database/lojas e senhas.xlsx
+++ b/database/lojas e senhas.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Desktop\TeleFluxo_Instalador\database\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E30C378-9F9D-4CE9-B2CE-B1D97D0BB0FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D2D62B0-19BA-4BED-AF64-159956C488BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{DC387A1A-0365-4EFE-8541-627FD66421E4}"/>
+    <workbookView xWindow="2250" yWindow="2250" windowWidth="21600" windowHeight="11295" xr2:uid="{DC387A1A-0365-4EFE-8541-627FD66421E4}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha4" sheetId="1" r:id="rId1"/>
@@ -412,7 +412,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -437,9 +437,6 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1042,7 +1039,7 @@
       <c r="F13" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="H13" s="10" t="s">
+      <c r="H13" s="7" t="s">
         <v>85</v>
       </c>
     </row>

</xml_diff>